<commit_message>
Drop Products, Stock Reports, Stock Lines and Targets from the AppSheet template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PEGfKnH6SrFsiNoNZ67yhb
</commit_message>
<xml_diff>
--- a/appsheet/Bengal2026_AppSheet_Template.xlsx
+++ b/appsheet/Bengal2026_AppSheet_Template.xlsx
@@ -12,18 +12,14 @@
     <sheet name="Areas" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Companies" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Brands" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Products" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Staff" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Customers" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Farmers" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Transactions" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Field Visits" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Stock Reports" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Stock Lines" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Leave Requests" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Targets" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Messages" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Company Pay" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Staff" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Customers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Farmers" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Transactions" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Field Visits" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Leave Requests" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Messages" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Company Pay" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -206,51 +202,6 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>One row per visit. Visit Type: Farmer Visit / Dealer Visit / Office Work.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Template</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Header of a stock check at a dealer.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment12.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Template</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Products counted in a stock report.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment13.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Template</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
         <t>Status: Pending / Approved / Rejected / Cancelled. Only managers/admins set Approved or Rejected.</t>
       </text>
     </comment>
@@ -258,22 +209,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment14.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Template</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Collection target per staff per period.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment11.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Template</author>
@@ -288,7 +224,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment12.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Template</author>
@@ -356,21 +292,6 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Product catalogue.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Template</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
         <t>Email = the Google account each person signs in with. Role: Admin / Manager / Field / Office.</t>
       </text>
     </comment>
@@ -378,7 +299,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Template</author>
@@ -393,7 +314,7 @@
 </comments>
 </file>
 
-<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments/comment7.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Template</author>
@@ -408,6 +329,21 @@
 </comments>
 </file>
 
+<file path=xl/comments/comment8.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Template</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Single ledger (replaces Entries + Statements). Amount is always positive; the app decides debit/credit from Txn Type.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/comments/comment9.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
@@ -416,7 +352,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Single ledger (replaces Entries + Statements). Amount is always positive; the app decides debit/credit from Txn Type.</t>
+        <t>One row per visit. Visit Type: Farmer Visit / Dealer Visit / Office Work.</t>
       </text>
     </comment>
   </commentList>
@@ -712,7 +648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -844,142 +780,94 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Products</t>
+          <t>Staff</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Product catalogue.</t>
+          <t>Email = the Google account each person signs in with. Role: Admin / Manager / Field / Office.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Staff</t>
+          <t>Customers</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Email = the Google account each person signs in with. Role: Admin / Manager / Field / Office.</t>
+          <t>Dealers/shops. Assigned Staff = one or more staff emails separated by ' , '.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Customers</t>
+          <t>Farmers</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Dealers/shops. Assigned Staff = one or more staff emails separated by ' , '.</t>
+          <t>Farmer master list (replaces New Farmer).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Farmers</t>
+          <t>Transactions</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Farmer master list (replaces New Farmer).</t>
+          <t>Single ledger (replaces Entries + Statements). Amount is always positive; the app decides debit/credit from Txn Type.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Transactions</t>
+          <t>Field Visits</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Single ledger (replaces Entries + Statements). Amount is always positive; the app decides debit/credit from Txn Type.</t>
+          <t>One row per visit. Visit Type: Farmer Visit / Dealer Visit / Office Work.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Field Visits</t>
+          <t>Leave Requests</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>One row per visit. Visit Type: Farmer Visit / Dealer Visit / Office Work.</t>
+          <t>Status: Pending / Approved / Rejected / Cancelled. Only managers/admins set Approved or Rejected.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Stock Reports</t>
+          <t>Messages</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Header of a stock check at a dealer.</t>
+          <t>Broadcasts + festive messages. Audience: All / Area / Selected. Status: Draft / Scheduled / Sent.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Stock Lines</t>
+          <t>Company Pay</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Products counted in a stock report.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Leave Requests</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Status: Pending / Approved / Rejected / Cancelled. Only managers/admins set Approved or Rejected.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Targets</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Collection target per staff per period.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Messages</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Broadcasts + festive messages. Audience: All / Area / Selected. Status: Draft / Scheduled / Sent.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Company Pay</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Company receipts/payments (admin only).</t>
         </is>
@@ -991,152 +879,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Txn ID</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Customer ID</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Brand</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Txn Type</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Invoice No</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>MRP Value</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
-        <is>
-          <t>Entered By</t>
-        </is>
-      </c>
-      <c r="L1" s="5" t="inlineStr">
-        <is>
-          <t>Entered At</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>T0001</t>
-        </is>
-      </c>
-      <c r="B2" s="9" t="n">
-        <v>46296</v>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>C0001</t>
-        </is>
-      </c>
-      <c r="D2" s="8" t="inlineStr">
-        <is>
-          <t>Microl</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>Microl Aqua</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>Sale</t>
-        </is>
-      </c>
-      <c r="G2" s="8" t="inlineStr">
-        <is>
-          <t>INV-1001</t>
-        </is>
-      </c>
-      <c r="H2" s="8" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I2" s="8" t="n">
-        <v>6000</v>
-      </c>
-      <c r="J2" s="8" t="inlineStr"/>
-      <c r="K2" s="8" t="inlineStr">
-        <is>
-          <t>you@example.com</t>
-        </is>
-      </c>
-      <c r="L2" s="10" t="n">
-        <v>46296.45833333334</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Sale,Payment,Stock Return,JV,Opening Balance"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1302,151 +1044,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Report ID</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Staff Email</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Report Date</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Customer ID</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Photo</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>S0001</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>you@example.com</t>
-        </is>
-      </c>
-      <c r="C2" s="9" t="n">
-        <v>46296</v>
-      </c>
-      <c r="D2" s="8" t="inlineStr">
-        <is>
-          <t>C0001</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="inlineStr"/>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>Monthly stock check</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Line ID</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Report ID</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>L0001</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>S0001</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>Example Product 1L</t>
-        </is>
-      </c>
-      <c r="D2" s="8" t="n">
-        <v>24</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1578,99 +1176,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Target ID</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Staff Email</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Period Name</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>End Date</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Target Amount</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Set By</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>TG0001</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>you@example.com</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>Oct-Dec 2026</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="n">
-        <v>46296</v>
-      </c>
-      <c r="E2" s="9" t="n">
-        <v>46387</v>
-      </c>
-      <c r="F2" s="8" t="n">
-        <v>500000</v>
-      </c>
-      <c r="G2" s="8" t="inlineStr">
-        <is>
-          <t>you@example.com</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1788,7 +1294,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2134,67 +1640,6 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Brand</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>MRP</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
-        <is>
-          <t>Example Product 1L</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>Microl Aqua</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="n">
-        <v>450</v>
-      </c>
-      <c r="D2" s="8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2316,7 +1761,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2428,7 +1873,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2569,4 +2014,150 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Txn ID</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Customer ID</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Txn Type</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Invoice No</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>MRP Value</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Entered By</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>Entered At</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>T0001</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="n">
+        <v>46296</v>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>C0001</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Microl</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>Microl Aqua</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>INV-1001</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J2" s="8" t="inlineStr"/>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>you@example.com</t>
+        </is>
+      </c>
+      <c r="L2" s="10" t="n">
+        <v>46296.45833333334</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sale,Payment,Stock Return,JV,Opening Balance"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
 </file>
</xml_diff>